<commit_message>
UPDATE SATURDAY 7 FEB 2026 16:03
</commit_message>
<xml_diff>
--- a/JANUARY 2026/FLOOR JANUARY 2026.xlsx
+++ b/JANUARY 2026/FLOOR JANUARY 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17020" activeTab="2"/>
+    <workbookView windowWidth="15980" windowHeight="17020" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -31,65 +31,8 @@
 </workbook>
 </file>
 
-<file path=xl/cellimages.xml><?xml version="1.0" encoding="utf-8"?>
-<etc:cellImages xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <etc:cellImage>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="ID_31806598E3BE46E18B6412FBA460C9ED" descr="PHOTO-2026-01-06-00-43-33"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:srcRect l="1066" t="8123" r="5377" b="14876"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8643620" y="1784985"/>
-          <a:ext cx="5292725" cy="7767320"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-  </etc:cellImage>
-  <etc:cellImage>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="ID_4148B145FB8D4C0AA5B41BE69295E076" descr="PHOTO-2026-01-06-18-10-09"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:srcRect l="2053" t="8978" r="4285" b="18807"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6587490" y="1823720"/>
-          <a:ext cx="5295265" cy="7528560"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-  </etc:cellImage>
-</etc:cellImages>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="43">
   <si>
     <t>DATE</t>
   </si>
@@ -127,6 +70,42 @@
     <t>GRAND TOTAL</t>
   </si>
   <si>
+    <t>0481/JL/UTM/0126</t>
+  </si>
+  <si>
+    <t>BLACK PLASTIC TRASH BAG 90X100 50 PCS</t>
+  </si>
+  <si>
+    <t>VACCUUM PLASTIC 16X25 100 PCS</t>
+  </si>
+  <si>
+    <t>DISHWASING SPONGE POLITEX 12 PCS</t>
+  </si>
+  <si>
+    <t>DISHWASHING WIRE POLITEX 12 PCS</t>
+  </si>
+  <si>
+    <t>0505/JL/UTM/0126</t>
+  </si>
+  <si>
+    <t>PLASTIC WRAP BESTCLING 45</t>
+  </si>
+  <si>
+    <t>BAKING PAPER CHEFFY 45X75</t>
+  </si>
+  <si>
+    <t>0635/JL/UTM/0126</t>
+  </si>
+  <si>
+    <t>CUP INJECTION 400ML + LID 25 PCS</t>
+  </si>
+  <si>
+    <t>0891/JL/UTM/0126</t>
+  </si>
+  <si>
+    <t>THERMAL PAPER 80X80</t>
+  </si>
+  <si>
     <t>SO05LC2601000210/00</t>
   </si>
   <si>
@@ -142,13 +121,22 @@
     <t>PPh 22</t>
   </si>
   <si>
-    <t>STATUS</t>
+    <t>SO05LC2601001612/00</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
   </si>
   <si>
     <t>QTY</t>
+  </si>
+  <si>
+    <t>DISHY 5L DISHWAHING</t>
+  </si>
+  <si>
+    <t>FLOOR CLEANER 5L</t>
+  </si>
+  <si>
+    <t>DETERGEN 5L</t>
   </si>
   <si>
     <t>NO</t>
@@ -186,8 +174,8 @@
     <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="180" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="181" formatCode="[$-409]d\-mmm\-yyyy;@"/>
-    <numFmt numFmtId="182" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="183" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="182" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="183" formatCode="dd\-mmm"/>
     <numFmt numFmtId="184" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="185" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??.00_-;_-@_-"/>
   </numFmts>
@@ -655,7 +643,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -670,72 +658,6 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -782,8 +704,34 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -812,6 +760,17 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -936,7 +895,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -948,34 +907,34 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1060,7 +1019,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1095,133 +1054,139 @@
     <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="181" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="181" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="181" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="3" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="180" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="181" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1230,78 +1195,69 @@
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="183" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="8" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="180" fontId="8" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1310,6 +1266,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1317,67 +1276,76 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1389,25 +1357,25 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="9" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1416,7 +1384,7 @@
     <xf numFmtId="180" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="182" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1481,6 +1449,415 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>27305</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2639695</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1252220</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="ID_1CACBEEAF13042EB8ABD4CB52304E3D5" descr="PHOTO-2026-01-06-00-43-33"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect l="1066" t="8123" r="5377" b="14876"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7240905" y="230505"/>
+          <a:ext cx="2563495" cy="3764915"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>27622</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>68262</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4774247</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>773112</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="ID_38097F0E6E864F92AC27F1E27852D20F" descr="PHOTO-2026-01-17-17-48-57"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect t="9999" b="3718"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8827135" y="-511175"/>
+          <a:ext cx="3181350" cy="4745990"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>85407</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>26987</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4717097</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>1447482</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="ID_1C5E43C2C367453BAF2826CB57A5A327" descr="PHOTO-2026-01-17-17-48-31"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:srcRect t="9990" b="3160"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8977630" y="2656205"/>
+          <a:ext cx="2880995" cy="4631690"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>35560</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>27305</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4766945</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>2945130</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="ID_1D13B2269DFB4942B24EE5BA96E02809" descr="PHOTO-2026-01-23-17-32-18"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:srcRect t="8421"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="8959850" y="5546725"/>
+          <a:ext cx="2917825" cy="4731385"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>46037</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>26987</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4755832</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>2672397</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="ID_FBA15014105644B68C8BFC203F1C7EBF" descr="PHOTO-2026-01-31-16-45-58"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="9095105" y="8381365"/>
+          <a:ext cx="2645410" cy="4709795"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>323215</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2505710</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>1557655</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="ID_4148B145FB8D4C0AA5B41BE69295E076" descr="PHOTO-2026-01-06-18-10-09"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect l="2053" t="8978" r="4285" b="18807"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6337300" y="226060"/>
+          <a:ext cx="2182495" cy="3103245"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>405765</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2423160</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>1557655</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="ID_F56F647980514D549FEA21F86BDFDD2C" descr="PHOTO-2026-01-15-16-18-58"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:srcRect t="11786" r="1201" b="7827"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6419850" y="4216400"/>
+          <a:ext cx="2017395" cy="3103245"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>51752</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>32067</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5301932</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>3783647</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="ID_49CAC5DC2B964E078E63224E751D9B0B" descr="PHOTO-2026-01-03-19-34-37"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect l="5123" t="17788" r="1745" b="8446"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="7452360" y="-272415"/>
+          <a:ext cx="3751580" cy="5249545"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>52070</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5302885</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1214755</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="ID_071A0DB504414623971F6BBE2D171133" descr="PHOTO-2026-01-15-16-43-00"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:srcRect t="15793" b="3577"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="7482205" y="3547110"/>
+          <a:ext cx="3693795" cy="5250815"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>47307</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>31432</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5306377</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>3706177</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="ID_753D150AAEEB4E189E512D64EC604A5E" descr="PHOTO-2026-01-23-19-31-50"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:srcRect t="13012" b="5676"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="16200000">
+          <a:off x="7490460" y="7313295"/>
+          <a:ext cx="3674745" cy="5259070"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1747,7 +2124,7 @@
     <col min="1" max="1" width="17.4296875" style="89"/>
     <col min="2" max="2" width="13.4296875" style="89" customWidth="1"/>
     <col min="3" max="3" width="36" style="89" customWidth="1"/>
-    <col min="4" max="4" width="21.2890625" style="88" customWidth="1"/>
+    <col min="4" max="4" width="21.2890625" style="87" customWidth="1"/>
     <col min="5" max="5" width="33.2890625" style="89" customWidth="1"/>
     <col min="6" max="6" width="17.2890625" style="89" customWidth="1"/>
     <col min="7" max="8" width="20.859375" style="89" customWidth="1"/>
@@ -1756,193 +2133,190 @@
     <col min="11" max="16384" width="18.0390625" style="89"/>
   </cols>
   <sheetData>
-    <row r="1" s="87" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="114" t="s">
+    <row r="1" s="86" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="117" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="115" t="s">
+      <c r="B1" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="115" t="s">
+      <c r="C1" s="118" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="115" t="s">
+      <c r="D1" s="118" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="115" t="s">
+      <c r="E1" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="115" t="s">
+      <c r="F1" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="115" t="s">
+      <c r="G1" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="115" t="s">
+      <c r="H1" s="118" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="87" customFormat="1" ht="60" customHeight="1" spans="1:10">
-      <c r="A2" s="96">
+    <row r="2" s="86" customFormat="1" ht="100" customHeight="1" spans="1:10">
+      <c r="A2" s="93">
         <v>46027</v>
       </c>
-      <c r="B2" s="93">
+      <c r="B2" s="104">
         <v>2963</v>
       </c>
-      <c r="C2" s="116" t="s">
+      <c r="C2" s="119" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="117">
+      <c r="D2" s="120">
         <v>24</v>
       </c>
-      <c r="E2" s="104" t="str">
-        <f>_xlfn.DISPIMG("ID_31806598E3BE46E18B6412FBA460C9ED",1)</f>
-        <v>=DISPIMG("ID_31806598E3BE46E18B6412FBA460C9ED",1)</v>
-      </c>
-      <c r="F2" s="105">
+      <c r="E2" s="108"/>
+      <c r="F2" s="109">
         <v>4833.33</v>
       </c>
-      <c r="G2" s="107">
+      <c r="G2" s="111">
         <f t="shared" ref="G2:G9" si="0">SUM(D2*F2)</f>
         <v>115999.92</v>
       </c>
-      <c r="H2" s="107">
+      <c r="H2" s="111">
         <f>SUM(G2:G4)</f>
         <v>266999.88</v>
       </c>
-      <c r="J2" s="87">
+      <c r="J2" s="86">
         <f>116000/24</f>
         <v>4833.33333333333</v>
       </c>
     </row>
-    <row r="3" s="87" customFormat="1" ht="60" customHeight="1" spans="1:10">
-      <c r="A3" s="98"/>
-      <c r="B3" s="93"/>
-      <c r="C3" s="116" t="s">
+    <row r="3" s="86" customFormat="1" ht="100" customHeight="1" spans="1:10">
+      <c r="A3" s="97"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="119" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="117">
+      <c r="D3" s="120">
         <v>12</v>
       </c>
-      <c r="E3" s="108"/>
-      <c r="F3" s="105">
+      <c r="E3" s="112"/>
+      <c r="F3" s="109">
         <v>3833.33</v>
       </c>
-      <c r="G3" s="107">
+      <c r="G3" s="111">
         <f t="shared" si="0"/>
         <v>45999.96</v>
       </c>
-      <c r="H3" s="109"/>
-      <c r="J3" s="87">
+      <c r="H3" s="113"/>
+      <c r="J3" s="86">
         <f>46000/12</f>
         <v>3833.33333333333</v>
       </c>
     </row>
-    <row r="4" s="87" customFormat="1" ht="60" customHeight="1" spans="1:10">
-      <c r="A4" s="98"/>
-      <c r="B4" s="93"/>
-      <c r="C4" s="116" t="s">
+    <row r="4" s="86" customFormat="1" ht="100" customHeight="1" spans="1:10">
+      <c r="A4" s="97"/>
+      <c r="B4" s="104"/>
+      <c r="C4" s="119" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="117">
+      <c r="D4" s="120">
         <v>100</v>
       </c>
-      <c r="E4" s="108"/>
-      <c r="F4" s="105">
+      <c r="E4" s="112"/>
+      <c r="F4" s="109">
         <v>1050</v>
       </c>
-      <c r="G4" s="107">
+      <c r="G4" s="111">
         <f t="shared" si="0"/>
         <v>105000</v>
       </c>
-      <c r="H4" s="109"/>
-      <c r="J4" s="87">
+      <c r="H4" s="113"/>
+      <c r="J4" s="86">
         <f>105000/100</f>
         <v>1050</v>
       </c>
     </row>
-    <row r="5" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A5" s="96"/>
-      <c r="B5" s="97"/>
-      <c r="C5" s="95"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="104"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="107">
+    <row r="5" s="86" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A5" s="93"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="99"/>
+      <c r="D5" s="120"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="111"/>
+      <c r="G5" s="111">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="107">
+      <c r="H5" s="111">
         <f>SUM(G5:G8)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A6" s="98"/>
-      <c r="B6" s="99"/>
-      <c r="C6" s="93"/>
-      <c r="D6" s="93"/>
-      <c r="E6" s="108"/>
-      <c r="F6" s="122"/>
-      <c r="G6" s="107">
+    <row r="6" s="86" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A6" s="97"/>
+      <c r="B6" s="98"/>
+      <c r="C6" s="104"/>
+      <c r="D6" s="104"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="125"/>
+      <c r="G6" s="111">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="109"/>
-    </row>
-    <row r="7" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A7" s="98"/>
-      <c r="B7" s="99"/>
-      <c r="C7" s="93"/>
-      <c r="D7" s="93"/>
-      <c r="E7" s="108"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="107">
+      <c r="H6" s="113"/>
+    </row>
+    <row r="7" s="86" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A7" s="97"/>
+      <c r="B7" s="98"/>
+      <c r="C7" s="104"/>
+      <c r="D7" s="104"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="111">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="109"/>
-    </row>
-    <row r="8" s="87" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
-      <c r="A8" s="98"/>
-      <c r="B8" s="99"/>
-      <c r="C8" s="97"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="108"/>
-      <c r="F8" s="122"/>
-      <c r="G8" s="107">
+      <c r="H7" s="113"/>
+    </row>
+    <row r="8" s="86" customFormat="1" ht="64.3" customHeight="1" spans="1:8">
+      <c r="A8" s="97"/>
+      <c r="B8" s="98"/>
+      <c r="C8" s="94"/>
+      <c r="D8" s="94"/>
+      <c r="E8" s="112"/>
+      <c r="F8" s="125"/>
+      <c r="G8" s="111">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="109"/>
-    </row>
-    <row r="9" s="87" customFormat="1" ht="258" customHeight="1" spans="1:8">
-      <c r="A9" s="92"/>
-      <c r="B9" s="93"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="112"/>
-      <c r="F9" s="123"/>
-      <c r="G9" s="105">
+      <c r="H8" s="113"/>
+    </row>
+    <row r="9" s="86" customFormat="1" ht="258" customHeight="1" spans="1:8">
+      <c r="A9" s="102"/>
+      <c r="B9" s="104"/>
+      <c r="C9" s="104"/>
+      <c r="D9" s="104"/>
+      <c r="E9" s="115"/>
+      <c r="F9" s="126"/>
+      <c r="G9" s="109">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H9" s="105">
+      <c r="H9" s="109">
         <f>SUM(G9)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" s="87" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A10" s="118" t="s">
+    <row r="10" s="86" customFormat="1" ht="18" customHeight="1" spans="1:8">
+      <c r="A10" s="121" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="119"/>
-      <c r="C10" s="120"/>
-      <c r="D10" s="121"/>
-      <c r="E10" s="124"/>
-      <c r="F10" s="124"/>
-      <c r="G10" s="125"/>
-      <c r="H10" s="126">
+      <c r="B10" s="122"/>
+      <c r="C10" s="123"/>
+      <c r="D10" s="124"/>
+      <c r="E10" s="127"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="128"/>
+      <c r="H10" s="129">
         <f>SUM(H2:H9)</f>
         <v>266999.88</v>
       </c>
@@ -1961,19 +2335,20 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelRow="7" outlineLevelCol="7"/>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="19.859375" style="88"/>
-    <col min="2" max="2" width="18.859375" style="88" customWidth="1"/>
+    <col min="1" max="1" width="19.859375" style="87"/>
+    <col min="2" max="2" width="21.3125" style="87" customWidth="1"/>
     <col min="3" max="3" width="43.0390625" style="88" customWidth="1"/>
-    <col min="4" max="4" width="14.4296875" style="88" customWidth="1"/>
+    <col min="4" max="4" width="14.4296875" style="87" customWidth="1"/>
     <col min="5" max="5" width="58.9609375" style="89" customWidth="1"/>
     <col min="6" max="6" width="19.5234375" style="89" customWidth="1"/>
     <col min="7" max="8" width="20.859375" style="89" customWidth="1"/>
@@ -1981,14 +2356,14 @@
     <col min="10" max="16384" width="9.140625" style="89"/>
   </cols>
   <sheetData>
-    <row r="1" s="87" customFormat="1" ht="16" customHeight="1" spans="1:8">
+    <row r="1" s="86" customFormat="1" ht="16" customHeight="1" spans="1:8">
       <c r="A1" s="90" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="91" t="s">
+      <c r="C1" s="92" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="91" t="s">
@@ -2007,113 +2382,237 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="87" customFormat="1" ht="249.35" customHeight="1" spans="1:8">
-      <c r="A2" s="92"/>
-      <c r="B2" s="93"/>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="106">
-        <f>D2*F2</f>
+    <row r="2" s="86" customFormat="1" ht="65" customHeight="1" spans="1:8">
+      <c r="A2" s="93">
+        <v>46038</v>
+      </c>
+      <c r="B2" s="94" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="96">
+        <v>9</v>
+      </c>
+      <c r="E2" s="108"/>
+      <c r="F2" s="109">
+        <v>50000</v>
+      </c>
+      <c r="G2" s="110">
+        <f t="shared" ref="G2:G10" si="0">D2*F2</f>
+        <v>450000</v>
+      </c>
+      <c r="H2" s="111">
+        <f>SUM(G2:G5)</f>
+        <v>1969000</v>
+      </c>
+    </row>
+    <row r="3" s="86" customFormat="1" ht="65" customHeight="1" spans="1:8">
+      <c r="A3" s="97"/>
+      <c r="B3" s="98"/>
+      <c r="C3" s="99" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="96">
+        <v>20</v>
+      </c>
+      <c r="E3" s="112"/>
+      <c r="F3" s="110">
+        <v>65000</v>
+      </c>
+      <c r="G3" s="110">
+        <f t="shared" si="0"/>
+        <v>1300000</v>
+      </c>
+      <c r="H3" s="113"/>
+    </row>
+    <row r="4" s="86" customFormat="1" ht="65" customHeight="1" spans="1:8">
+      <c r="A4" s="97"/>
+      <c r="B4" s="98"/>
+      <c r="C4" s="99" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="96">
+        <v>3</v>
+      </c>
+      <c r="E4" s="112"/>
+      <c r="F4" s="110">
+        <v>38000</v>
+      </c>
+      <c r="G4" s="110">
+        <f t="shared" si="0"/>
+        <v>114000</v>
+      </c>
+      <c r="H4" s="113"/>
+    </row>
+    <row r="5" s="86" customFormat="1" ht="65" customHeight="1" spans="1:8">
+      <c r="A5" s="100"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="99" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="96">
+        <v>3</v>
+      </c>
+      <c r="E5" s="112"/>
+      <c r="F5" s="110">
+        <v>35000</v>
+      </c>
+      <c r="G5" s="110">
+        <f t="shared" si="0"/>
+        <v>105000</v>
+      </c>
+      <c r="H5" s="113"/>
+    </row>
+    <row r="6" s="86" customFormat="1" ht="115" customHeight="1" spans="1:8">
+      <c r="A6" s="93">
+        <v>46039</v>
+      </c>
+      <c r="B6" s="94" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="99" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="96">
+        <v>10</v>
+      </c>
+      <c r="E6" s="108"/>
+      <c r="F6" s="110">
+        <v>165000</v>
+      </c>
+      <c r="G6" s="110">
+        <f t="shared" si="0"/>
+        <v>1650000</v>
+      </c>
+      <c r="H6" s="111">
+        <f>SUM(G6:G7)</f>
+        <v>2650000</v>
+      </c>
+    </row>
+    <row r="7" s="86" customFormat="1" ht="115" customHeight="1" spans="1:8">
+      <c r="A7" s="97"/>
+      <c r="B7" s="98"/>
+      <c r="C7" s="99" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="96">
+        <v>5</v>
+      </c>
+      <c r="E7" s="112"/>
+      <c r="F7" s="110">
+        <v>200000</v>
+      </c>
+      <c r="G7" s="110">
+        <f t="shared" si="0"/>
+        <v>1000000</v>
+      </c>
+      <c r="H7" s="113"/>
+    </row>
+    <row r="8" s="86" customFormat="1" ht="233.15" customHeight="1" spans="1:8">
+      <c r="A8" s="102">
+        <v>46044</v>
+      </c>
+      <c r="B8" s="103" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="99" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="96">
+        <v>20</v>
+      </c>
+      <c r="E8" s="114"/>
+      <c r="F8" s="110">
+        <v>35000</v>
+      </c>
+      <c r="G8" s="110">
+        <f t="shared" si="0"/>
+        <v>700000</v>
+      </c>
+      <c r="H8" s="110">
+        <f>SUM(G8)</f>
+        <v>700000</v>
+      </c>
+    </row>
+    <row r="9" s="86" customFormat="1" ht="212.5" customHeight="1" spans="1:8">
+      <c r="A9" s="102">
+        <v>46053</v>
+      </c>
+      <c r="B9" s="103" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="99" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="96">
+        <v>1</v>
+      </c>
+      <c r="E9" s="114"/>
+      <c r="F9" s="109">
+        <v>780000</v>
+      </c>
+      <c r="G9" s="110">
+        <f t="shared" si="0"/>
+        <v>780000</v>
+      </c>
+      <c r="H9" s="110">
+        <f>SUM(G9)</f>
+        <v>780000</v>
+      </c>
+    </row>
+    <row r="10" s="86" customFormat="1" ht="83" customHeight="1" spans="1:8">
+      <c r="A10" s="102"/>
+      <c r="B10" s="103"/>
+      <c r="C10" s="99"/>
+      <c r="D10" s="96"/>
+      <c r="E10" s="114"/>
+      <c r="F10" s="109"/>
+      <c r="G10" s="110">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H2" s="105">
-        <f>SUM(G2:G2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" s="87" customFormat="1" ht="251.35" customHeight="1" spans="1:8">
-      <c r="A3" s="92"/>
-      <c r="B3" s="93"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="94"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="106"/>
-      <c r="G3" s="106">
-        <f>D3*F3</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="107">
-        <f>SUM(G3:G3)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" s="87" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A4" s="96"/>
-      <c r="B4" s="97"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="94"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="106"/>
-      <c r="G4" s="106">
-        <f>D4*F4</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="107">
-        <f>SUM(G4:G6)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" s="87" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A5" s="98"/>
-      <c r="B5" s="99"/>
-      <c r="C5" s="95"/>
-      <c r="D5" s="100"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="106">
-        <f>D5*F5</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="109"/>
-    </row>
-    <row r="6" s="87" customFormat="1" ht="83" customHeight="1" spans="1:8">
-      <c r="A6" s="101"/>
-      <c r="B6" s="102"/>
-      <c r="C6" s="95"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="110"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="106">
-        <f>D6*F6</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="111"/>
-    </row>
-    <row r="7" s="87" customFormat="1" ht="200" customHeight="1" spans="1:8">
-      <c r="A7" s="92"/>
-      <c r="B7" s="93"/>
-      <c r="C7" s="95"/>
-      <c r="D7" s="100"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="107"/>
-      <c r="G7" s="107"/>
-      <c r="H7" s="105"/>
-    </row>
-    <row r="8" s="87" customFormat="1" spans="1:8">
-      <c r="A8" s="103"/>
-      <c r="B8" s="103"/>
-      <c r="C8" s="103"/>
-      <c r="D8" s="103"/>
-      <c r="E8" s="103"/>
-      <c r="F8" s="103"/>
-      <c r="G8" s="113"/>
-      <c r="H8" s="113">
-        <f>SUM(H2:H7)</f>
-        <v>0</v>
+      <c r="H10" s="110"/>
+    </row>
+    <row r="11" s="86" customFormat="1" ht="200" customHeight="1" spans="1:8">
+      <c r="A11" s="102"/>
+      <c r="B11" s="104"/>
+      <c r="C11" s="99"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="115"/>
+      <c r="F11" s="111"/>
+      <c r="G11" s="111"/>
+      <c r="H11" s="109"/>
+    </row>
+    <row r="12" s="86" customFormat="1" spans="1:8">
+      <c r="A12" s="106"/>
+      <c r="B12" s="106"/>
+      <c r="C12" s="107"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="106"/>
+      <c r="F12" s="106"/>
+      <c r="G12" s="116"/>
+      <c r="H12" s="116">
+        <f>SUM(H2:H11)</f>
+        <v>6099000</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A4:A6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="H4:H6"/>
+  <mergeCells count="9">
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="H6:H7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2133,45 +2632,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="D1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="51" t="s">
+      <c r="E1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="F1" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="G1" s="53" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A2" s="52">
+      <c r="A2" s="46">
         <v>46027</v>
       </c>
-      <c r="B2" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="53" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="54">
+      <c r="B2" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="56">
         <v>80</v>
       </c>
-      <c r="E2" s="73" t="str">
-        <f>_xlfn.DISPIMG("ID_4148B145FB8D4C0AA5B41BE69295E076",1)</f>
-        <v>=DISPIMG("ID_4148B145FB8D4C0AA5B41BE69295E076",1)</v>
-      </c>
+      <c r="E2" s="73"/>
       <c r="F2" s="74">
         <v>6063.9632</v>
       </c>
@@ -2181,62 +2677,62 @@
       </c>
     </row>
     <row r="3" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A3" s="52"/>
-      <c r="B3" s="39"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="56"/>
+      <c r="A3" s="46"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="58"/>
       <c r="E3" s="73"/>
       <c r="F3" s="76"/>
       <c r="G3" s="75"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="52"/>
-      <c r="B4" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58">
+      <c r="A4" s="46"/>
+      <c r="B4" s="59" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="59"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60">
         <f>SUM(G2:G3)</f>
         <v>485117.056</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="52"/>
-      <c r="B5" s="57" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58">
+      <c r="A5" s="46"/>
+      <c r="B5" s="59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="59"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60">
         <f>G4*11%</f>
         <v>53362.87616</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="52"/>
-      <c r="B6" s="57" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="57"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
+      <c r="A6" s="46"/>
+      <c r="B6" s="59" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="59"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="77">
         <v>485.12</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="52"/>
-      <c r="B7" s="57" t="s">
+      <c r="A7" s="46"/>
+      <c r="B7" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="57"/>
-      <c r="D7" s="58"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="60"/>
       <c r="E7" s="78"/>
       <c r="F7" s="78"/>
       <c r="G7" s="78">
@@ -2245,58 +2741,76 @@
       </c>
     </row>
     <row r="8" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A8" s="52"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="61"/>
+      <c r="A8" s="46">
+        <v>46036</v>
+      </c>
+      <c r="B8" s="61" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="56">
+        <v>100</v>
+      </c>
       <c r="E8" s="79"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="80"/>
+      <c r="F8" s="74">
+        <v>6063963.9632</v>
+      </c>
+      <c r="G8" s="75">
+        <f>F8*D8</f>
+        <v>606396396.32</v>
+      </c>
     </row>
     <row r="9" ht="123.5" customHeight="1" spans="1:7">
-      <c r="A9" s="52"/>
+      <c r="A9" s="46"/>
       <c r="B9" s="62"/>
-      <c r="C9" s="60"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="81"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="80"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="58"/>
+      <c r="E9" s="80"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="75"/>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="63"/>
-      <c r="B10" s="57" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="57"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="82"/>
-      <c r="F10" s="58"/>
-      <c r="G10" s="58">
+      <c r="B10" s="59" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="59"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="81"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60">
         <f>SUM(G8:G9)</f>
-        <v>0</v>
+        <v>606396396.32</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="64"/>
       <c r="B11" s="65" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C11" s="66"/>
-      <c r="D11" s="58"/>
-      <c r="E11" s="82"/>
-      <c r="F11" s="58"/>
-      <c r="G11" s="58"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60">
+        <f>G10*11%</f>
+        <v>66703603.5952</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="63"/>
-      <c r="B12" s="57" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="57"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="82"/>
-      <c r="F12" s="58"/>
-      <c r="G12" s="77"/>
+      <c r="B12" s="59" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="59"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="81"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="77">
+        <v>606.4</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="67"/>
@@ -2304,12 +2818,11 @@
         <v>7</v>
       </c>
       <c r="C13" s="69"/>
-      <c r="D13" s="58"/>
+      <c r="D13" s="60"/>
       <c r="E13" s="78"/>
-      <c r="F13" s="83"/>
+      <c r="F13" s="82"/>
       <c r="G13" s="78">
-        <f>SUM(G10:G12)</f>
-        <v>0</v>
+        <v>673706.31</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2319,15 +2832,15 @@
       <c r="B14" s="71"/>
       <c r="C14" s="71"/>
       <c r="D14" s="72"/>
-      <c r="E14" s="84">
+      <c r="E14" s="83">
         <f>G7+G13</f>
-        <v>538965.05216</v>
-      </c>
-      <c r="F14" s="85"/>
-      <c r="G14" s="86"/>
+        <v>1212671.36216</v>
+      </c>
+      <c r="F14" s="84"/>
+      <c r="G14" s="85"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="24">
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
@@ -2343,276 +2856,378 @@
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C8:C9"/>
     <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D8:D9"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="E8:E9"/>
     <mergeCell ref="F2:F3"/>
+    <mergeCell ref="F8:F9"/>
     <mergeCell ref="G2:G3"/>
+    <mergeCell ref="G8:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="4"/>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="12" customWidth="1"/>
-    <col min="2" max="2" width="12.6015625" style="36" customWidth="1"/>
-    <col min="3" max="3" width="36.125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="18.828125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="12.2890625" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="12"/>
+    <col min="1" max="1" width="11.9375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12.6015625" style="42" customWidth="1"/>
+    <col min="3" max="3" width="18.828125" style="12" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" s="35" customFormat="1" ht="19" customHeight="1" spans="1:5">
-      <c r="A1" s="37" t="s">
+    <row r="1" s="41" customFormat="1" ht="19" customHeight="1" spans="1:3">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="37" t="s">
+      <c r="C1" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="37" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
-      <c r="A2" s="39"/>
-      <c r="B2" s="40"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="41"/>
-    </row>
-    <row r="3" s="12" customFormat="1" ht="255.1" customHeight="1" spans="1:5">
-      <c r="A3" s="39"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="48"/>
-    </row>
-    <row r="4" s="12" customFormat="1" ht="249.95" customHeight="1" spans="1:5">
-      <c r="A4" s="39"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="48"/>
-    </row>
-    <row r="5" s="12" customFormat="1" ht="256.25" customHeight="1" spans="1:5">
-      <c r="A5" s="39"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="48"/>
-    </row>
-    <row r="6" s="12" customFormat="1" ht="253.85" customHeight="1" spans="1:5">
-      <c r="A6" s="39"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="48"/>
-    </row>
-    <row r="7" s="12" customFormat="1" ht="254.65" customHeight="1" spans="1:5">
-      <c r="A7" s="39"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="48"/>
-    </row>
-    <row r="8" s="12" customFormat="1" ht="255.35" customHeight="1" spans="1:5">
-      <c r="A8" s="39"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="48"/>
-    </row>
-    <row r="9" s="12" customFormat="1" ht="266.95" customHeight="1" spans="1:5">
-      <c r="A9" s="39"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="48"/>
-    </row>
-    <row r="10" s="12" customFormat="1" ht="261.95" customHeight="1" spans="1:5">
-      <c r="A10" s="39"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="48"/>
-    </row>
-    <row r="11" s="12" customFormat="1" ht="261.9" customHeight="1" spans="1:5">
-      <c r="A11" s="39"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="48"/>
-    </row>
-    <row r="12" s="12" customFormat="1" ht="270.7" customHeight="1" spans="1:5">
-      <c r="A12" s="39"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="48"/>
-    </row>
-    <row r="13" s="12" customFormat="1" ht="261.1" customHeight="1" spans="1:5">
-      <c r="A13" s="39"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="48"/>
-    </row>
-    <row r="14" s="12" customFormat="1" ht="257.15" customHeight="1" spans="1:5">
-      <c r="A14" s="39"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="48"/>
-    </row>
-    <row r="15" s="12" customFormat="1" ht="263.55" customHeight="1" spans="1:5">
-      <c r="A15" s="39"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="48"/>
-    </row>
-    <row r="16" s="12" customFormat="1" ht="270.35" customHeight="1" spans="1:5">
-      <c r="A16" s="39"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="48"/>
-    </row>
-    <row r="17" s="12" customFormat="1" ht="261.7" customHeight="1" spans="1:5">
-      <c r="A17" s="39"/>
-      <c r="B17" s="40"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="48"/>
-    </row>
-    <row r="18" s="12" customFormat="1" ht="260" customHeight="1" spans="1:5">
-      <c r="A18" s="39"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="48"/>
-    </row>
-    <row r="19" s="12" customFormat="1" ht="263.2" customHeight="1" spans="1:5">
-      <c r="A19" s="39"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="48"/>
-    </row>
-    <row r="20" s="12" customFormat="1" ht="289.95" customHeight="1" spans="1:5">
-      <c r="A20" s="39"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="48"/>
-    </row>
-    <row r="21" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A21" s="39"/>
-      <c r="B21" s="40"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="48"/>
-    </row>
-    <row r="22" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A22" s="39"/>
-      <c r="B22" s="40"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="48"/>
-    </row>
-    <row r="23" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A23" s="39"/>
-      <c r="B23" s="40"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="48"/>
-    </row>
-    <row r="24" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A24" s="39"/>
-      <c r="B24" s="40"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="41"/>
-    </row>
-    <row r="25" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A25" s="39"/>
-      <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="41"/>
-    </row>
-    <row r="26" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A26" s="39"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="41"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="41"/>
-    </row>
-    <row r="27" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A27" s="39">
-        <v>45960</v>
-      </c>
-      <c r="B27" s="40"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="41"/>
-    </row>
-    <row r="28" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A28" s="39">
-        <v>45961</v>
-      </c>
-      <c r="B28" s="40"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="42"/>
-      <c r="E28" s="41"/>
-    </row>
-    <row r="29" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A29" s="39"/>
-      <c r="B29" s="40"/>
-      <c r="C29" s="41"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="41"/>
-    </row>
-    <row r="30" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A30" s="39"/>
-      <c r="B30" s="40"/>
-      <c r="C30" s="41"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="41"/>
-    </row>
-    <row r="31" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A31" s="39"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="41"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="41"/>
-    </row>
-    <row r="32" s="12" customFormat="1" spans="1:5">
-      <c r="A32" s="44"/>
-      <c r="B32" s="45"/>
-      <c r="C32" s="46">
-        <f>SUM(D2:D31)</f>
-        <v>0</v>
-      </c>
-      <c r="D32" s="47"/>
-      <c r="E32" s="49"/>
+    </row>
+    <row r="2" s="12" customFormat="1" spans="1:3">
+      <c r="A2" s="46">
+        <v>46024</v>
+      </c>
+      <c r="B2" s="47">
+        <v>1462</v>
+      </c>
+      <c r="C2" s="48">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="3" s="12" customFormat="1" spans="1:3">
+      <c r="A3" s="46">
+        <v>46026</v>
+      </c>
+      <c r="B3" s="47">
+        <v>1463</v>
+      </c>
+      <c r="C3" s="49">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="4" s="12" customFormat="1" spans="1:3">
+      <c r="A4" s="46">
+        <v>46027</v>
+      </c>
+      <c r="B4" s="47">
+        <v>1464</v>
+      </c>
+      <c r="C4" s="49">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="5" s="12" customFormat="1" spans="1:3">
+      <c r="A5" s="46">
+        <v>46028</v>
+      </c>
+      <c r="B5" s="47">
+        <v>1465</v>
+      </c>
+      <c r="C5" s="49">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="6" s="12" customFormat="1" spans="1:3">
+      <c r="A6" s="46">
+        <v>46029</v>
+      </c>
+      <c r="B6" s="47">
+        <v>1466</v>
+      </c>
+      <c r="C6" s="49">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="7" s="12" customFormat="1" spans="1:3">
+      <c r="A7" s="46">
+        <v>46030</v>
+      </c>
+      <c r="B7" s="47">
+        <v>1467</v>
+      </c>
+      <c r="C7" s="49">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="8" s="12" customFormat="1" spans="1:3">
+      <c r="A8" s="46">
+        <v>46032</v>
+      </c>
+      <c r="B8" s="47">
+        <v>1468</v>
+      </c>
+      <c r="C8" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="9" s="12" customFormat="1" spans="1:3">
+      <c r="A9" s="46">
+        <v>46033</v>
+      </c>
+      <c r="B9" s="47">
+        <v>1469</v>
+      </c>
+      <c r="C9" s="49">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="10" s="12" customFormat="1" spans="1:3">
+      <c r="A10" s="46">
+        <v>46034</v>
+      </c>
+      <c r="B10" s="47">
+        <v>1470</v>
+      </c>
+      <c r="C10" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="11" s="12" customFormat="1" spans="1:3">
+      <c r="A11" s="46">
+        <v>46035</v>
+      </c>
+      <c r="B11" s="47">
+        <v>1471</v>
+      </c>
+      <c r="C11" s="49">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="12" s="12" customFormat="1" spans="1:3">
+      <c r="A12" s="46">
+        <v>46036</v>
+      </c>
+      <c r="B12" s="47">
+        <v>1472</v>
+      </c>
+      <c r="C12" s="49">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="13" s="12" customFormat="1" spans="1:3">
+      <c r="A13" s="46">
+        <v>46037</v>
+      </c>
+      <c r="B13" s="47">
+        <v>1473</v>
+      </c>
+      <c r="C13" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="14" s="12" customFormat="1" spans="1:3">
+      <c r="A14" s="46">
+        <v>46038</v>
+      </c>
+      <c r="B14" s="47">
+        <v>1474</v>
+      </c>
+      <c r="C14" s="49">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="15" s="12" customFormat="1" spans="1:3">
+      <c r="A15" s="46">
+        <v>46039</v>
+      </c>
+      <c r="B15" s="47">
+        <v>1475</v>
+      </c>
+      <c r="C15" s="49">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="16" s="12" customFormat="1" spans="1:3">
+      <c r="A16" s="46">
+        <v>46040</v>
+      </c>
+      <c r="B16" s="47">
+        <v>1476</v>
+      </c>
+      <c r="C16" s="49">
+        <v>72000</v>
+      </c>
+    </row>
+    <row r="17" s="12" customFormat="1" spans="1:3">
+      <c r="A17" s="46">
+        <v>46041</v>
+      </c>
+      <c r="B17" s="47">
+        <v>1477</v>
+      </c>
+      <c r="C17" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="18" s="12" customFormat="1" spans="1:3">
+      <c r="A18" s="46">
+        <v>46042</v>
+      </c>
+      <c r="B18" s="47">
+        <v>1478</v>
+      </c>
+      <c r="C18" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="19" s="12" customFormat="1" spans="1:3">
+      <c r="A19" s="46">
+        <v>46043</v>
+      </c>
+      <c r="B19" s="47">
+        <v>1479</v>
+      </c>
+      <c r="C19" s="49">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="20" s="12" customFormat="1" spans="1:3">
+      <c r="A20" s="46">
+        <v>46044</v>
+      </c>
+      <c r="B20" s="47">
+        <v>1480</v>
+      </c>
+      <c r="C20" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="21" s="12" customFormat="1" spans="1:3">
+      <c r="A21" s="46">
+        <v>46045</v>
+      </c>
+      <c r="B21" s="47">
+        <v>1481</v>
+      </c>
+      <c r="C21" s="49">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="22" s="12" customFormat="1" spans="1:3">
+      <c r="A22" s="46">
+        <v>46046</v>
+      </c>
+      <c r="B22" s="47">
+        <v>1482</v>
+      </c>
+      <c r="C22" s="49">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="23" s="12" customFormat="1" spans="1:3">
+      <c r="A23" s="46">
+        <v>46047</v>
+      </c>
+      <c r="B23" s="47">
+        <v>1483</v>
+      </c>
+      <c r="C23" s="49">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="24" s="12" customFormat="1" spans="1:3">
+      <c r="A24" s="46">
+        <v>46048</v>
+      </c>
+      <c r="B24" s="47">
+        <v>1484</v>
+      </c>
+      <c r="C24" s="48">
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="25" s="12" customFormat="1" spans="1:3">
+      <c r="A25" s="46">
+        <v>46049</v>
+      </c>
+      <c r="B25" s="47">
+        <v>1485</v>
+      </c>
+      <c r="C25" s="48">
+        <v>105000</v>
+      </c>
+    </row>
+    <row r="26" s="12" customFormat="1" spans="1:3">
+      <c r="A26" s="46">
+        <v>46050</v>
+      </c>
+      <c r="B26" s="47">
+        <v>1486</v>
+      </c>
+      <c r="C26" s="48">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="27" s="12" customFormat="1" spans="1:3">
+      <c r="A27" s="46">
+        <v>46051</v>
+      </c>
+      <c r="B27" s="47">
+        <v>1487</v>
+      </c>
+      <c r="C27" s="48">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="28" s="12" customFormat="1" spans="1:3">
+      <c r="A28" s="46">
+        <v>46052</v>
+      </c>
+      <c r="B28" s="47">
+        <v>1488</v>
+      </c>
+      <c r="C28" s="48">
+        <v>96000</v>
+      </c>
+    </row>
+    <row r="29" s="12" customFormat="1" spans="1:3">
+      <c r="A29" s="46">
+        <v>46053</v>
+      </c>
+      <c r="B29" s="47">
+        <v>1489</v>
+      </c>
+      <c r="C29" s="48">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="30" s="12" customFormat="1" spans="1:3">
+      <c r="A30" s="50" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="51"/>
+      <c r="C30" s="48">
+        <f>SUM(C1:C29)</f>
+        <v>1441000</v>
+      </c>
+    </row>
+    <row r="31" s="12" customFormat="1" spans="1:2">
+      <c r="A31" s="13"/>
+      <c r="B31" s="42"/>
+    </row>
+    <row r="32" s="12" customFormat="1" spans="1:2">
+      <c r="A32" s="13"/>
+      <c r="B32" s="42"/>
+    </row>
+    <row r="33" s="12" customFormat="1" spans="1:2">
+      <c r="A33" s="13"/>
+      <c r="B33" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
+  <mergeCells count="1">
+    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2622,113 +3237,223 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="6"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="21.140625" style="13" customWidth="1"/>
-    <col min="2" max="2" width="27.5703125" style="12" customWidth="1"/>
-    <col min="3" max="3" width="30.75" style="12" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="42.2890625" style="12" customWidth="1"/>
+    <col min="3" max="3" width="15.8359375" style="14" customWidth="1"/>
     <col min="4" max="4" width="65.703125" style="12" customWidth="1"/>
     <col min="5" max="7" width="32.3359375" style="12" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="12"/>
+    <col min="8" max="9" width="9.140625" style="12"/>
+    <col min="10" max="10" width="12.859375" style="12"/>
+    <col min="11" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" s="11" customFormat="1" ht="35" customHeight="1" spans="1:7">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="15" t="s">
+      <c r="B1" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="17" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="12" customFormat="1" ht="240.3" customHeight="1" spans="1:7">
-      <c r="A2" s="16"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="26">
-        <f>C2*E2</f>
+    <row r="2" s="12" customFormat="1" ht="300.8" customHeight="1" spans="1:7">
+      <c r="A2" s="18">
+        <v>46025</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="20">
+        <v>5</v>
+      </c>
+      <c r="D2" s="21"/>
+      <c r="E2" s="34">
+        <v>60000</v>
+      </c>
+      <c r="F2" s="34">
+        <f t="shared" ref="F2:F10" si="0">C2*E2</f>
+        <v>300000</v>
+      </c>
+      <c r="G2" s="34">
+        <f>SUM(F2:F2)</f>
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="3" s="12" customFormat="1" ht="100" customHeight="1" spans="1:7">
+      <c r="A3" s="22">
+        <v>46037</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="24">
+        <v>5</v>
+      </c>
+      <c r="D3" s="25"/>
+      <c r="E3" s="23">
+        <v>60000</v>
+      </c>
+      <c r="F3" s="34">
+        <f t="shared" si="0"/>
+        <v>300000</v>
+      </c>
+      <c r="G3" s="35">
+        <f>SUM(F3:F5)</f>
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="4" s="12" customFormat="1" ht="100" customHeight="1" spans="1:7">
+      <c r="A4" s="26"/>
+      <c r="B4" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="24">
+        <v>5</v>
+      </c>
+      <c r="D4" s="27"/>
+      <c r="E4" s="23">
+        <v>60000</v>
+      </c>
+      <c r="F4" s="34">
+        <f t="shared" si="0"/>
+        <v>300000</v>
+      </c>
+      <c r="G4" s="36"/>
+    </row>
+    <row r="5" s="12" customFormat="1" ht="100" customHeight="1" spans="1:7">
+      <c r="A5" s="28"/>
+      <c r="B5" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="24">
+        <v>3</v>
+      </c>
+      <c r="D5" s="29"/>
+      <c r="E5" s="23">
+        <v>55000</v>
+      </c>
+      <c r="F5" s="34">
+        <f t="shared" si="0"/>
+        <v>165000</v>
+      </c>
+      <c r="G5" s="37"/>
+    </row>
+    <row r="6" s="12" customFormat="1" ht="294.2" customHeight="1" spans="1:7">
+      <c r="A6" s="30">
+        <v>46045</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="24">
+        <v>6</v>
+      </c>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23">
+        <v>60000</v>
+      </c>
+      <c r="F6" s="34">
+        <f t="shared" si="0"/>
+        <v>360000</v>
+      </c>
+      <c r="G6" s="38">
+        <f>SUM(F6)</f>
+        <v>360000</v>
+      </c>
+    </row>
+    <row r="7" s="12" customFormat="1" ht="26" spans="1:7">
+      <c r="A7" s="30"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="34">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G2" s="27">
-        <f>SUM(F2:F2)</f>
+      <c r="G7" s="38"/>
+    </row>
+    <row r="8" s="12" customFormat="1" ht="26" spans="1:7">
+      <c r="A8" s="30"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="34">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
-      <c r="A3" s="20"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="30"/>
-    </row>
-    <row r="4" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
-      <c r="A4" s="20"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="31"/>
-    </row>
-    <row r="5" s="12" customFormat="1" ht="80" customHeight="1" spans="1:7">
-      <c r="A5" s="20"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="32"/>
-    </row>
-    <row r="6" s="12" customFormat="1" ht="26" spans="1:7">
-      <c r="A6" s="20"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="33"/>
-    </row>
-    <row r="7" s="12" customFormat="1" ht="39" customHeight="1" spans="1:7">
-      <c r="A7" s="20" t="s">
+      <c r="G8" s="38"/>
+    </row>
+    <row r="9" s="12" customFormat="1" ht="26" spans="1:7">
+      <c r="A9" s="30"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="34">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="38">
+        <f>SUM(F9:F10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" s="12" customFormat="1" ht="26" spans="1:7">
+      <c r="A10" s="30"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="34">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="38"/>
+    </row>
+    <row r="11" s="12" customFormat="1" ht="39" customHeight="1" spans="1:7">
+      <c r="A11" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="34">
-        <f>SUM(G2:G6)</f>
-        <v>0</v>
-      </c>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="39">
+        <f>SUM(G2:G10)</f>
+        <v>1425000</v>
+      </c>
+      <c r="F11" s="39"/>
+      <c r="G11" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="G3:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2745,13 +3470,13 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -2759,7 +3484,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H10</f>
@@ -2771,11 +3496,11 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C3" s="8">
-        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H8</f>
-        <v>0</v>
+        <f>'UD Abdi Jaya (Bag, Cup, Box)'!H12</f>
+        <v>6099000</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2783,11 +3508,11 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E14</f>
-        <v>538965.05216</v>
+        <v>1212671.36216</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2795,11 +3520,11 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="9">
-        <f>'Vickel Laundry'!C32</f>
-        <v>0</v>
+        <v>41</v>
+      </c>
+      <c r="C5" s="9" t="e">
+        <f>'Vickel Laundry'!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2807,7 +3532,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G7</f>
@@ -2819,9 +3544,9 @@
         <v>7</v>
       </c>
       <c r="B7" s="7"/>
-      <c r="C7" s="10">
+      <c r="C7" s="10" t="e">
         <f>SUM(C2:C5)</f>
-        <v>805964.93216</v>
+        <v>#REF!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>